<commit_message>
Added latest NASA files
</commit_message>
<xml_diff>
--- a/2024-05-04to05-10 (A5) C384400 NASA/02_CASimportExport/01_v01_Organizational Support Functions PLACE HOLDER.xlsx
+++ b/2024-05-04to05-10 (A5) C384400 NASA/02_CASimportExport/01_v01_Organizational Support Functions PLACE HOLDER.xlsx
@@ -32838,9 +32838,9 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001F513751AC33344AB32CFD2920EFE649" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="683516f7d70434a0e4dbd6c476be8d5b">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="72e3a154-4955-46c3-9573-e9dec3e1f195" xmlns:ns3="ec500478-62e0-46fc-87f1-cfa988e486b4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cf4a15c6a1eec5dbba94230cc6a50510" ns2:_="" ns3:_="">
-    <xsd:import namespace="72e3a154-4955-46c3-9573-e9dec3e1f195"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F041F74863103D4C9C3AA0A07291BB02" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="acfac7a7740a1b2d1a4bdbff0c117f3f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="25bcabcf-d275-4206-9fb1-2f2d419cd22b" xmlns:ns3="ec500478-62e0-46fc-87f1-cfa988e486b4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f1327b100fd5e593709bdd676db08f29" ns2:_="" ns3:_="">
+    <xsd:import namespace="25bcabcf-d275-4206-9fb1-2f2d419cd22b"/>
     <xsd:import namespace="ec500478-62e0-46fc-87f1-cfa988e486b4"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -32850,15 +32850,21 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -32866,7 +32872,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="72e3a154-4955-46c3-9573-e9dec3e1f195" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="25bcabcf-d275-4206-9fb1-2f2d419cd22b" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -32879,50 +32885,77 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="12" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceKeyPoints" ma:index="13" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoTags" ma:index="15" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="14" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="15" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7f35f27a-c890-4130-b78e-bbe546ff31bf" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="23" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ec500478-62e0-46fc-87f1-cfa988e486b4" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="16" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -32941,12 +32974,23 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="17" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="22" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{516b899e-718a-4501-bed1-5bdbb6269459}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ec500478-62e0-46fc-87f1-cfa988e486b4">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -33050,7 +33094,12 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="ec500478-62e0-46fc-87f1-cfa988e486b4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="25bcabcf-d275-4206-9fb1-2f2d419cd22b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
@@ -33063,22 +33112,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65ABCF49-6E27-483B-8280-D9598C75A60A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="72e3a154-4955-46c3-9573-e9dec3e1f195"/>
-    <ds:schemaRef ds:uri="ec500478-62e0-46fc-87f1-cfa988e486b4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BACCEF0E-3FD2-4362-8D4F-200690821C7B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>